<commit_message>
Release v1.3.8: command-line aliases, typed-point DRAW, and dockable terminal.
Ship the command registry (short form = full name), MOVE/ZOOM sessions, Atomik HELP, and version-archive Windows EXE.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ShyamGui/CHANGELOG.xlsx
+++ b/ShyamGui/CHANGELOG.xlsx
@@ -8,19 +8,20 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.7 Changes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.6 Changes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.5 Changes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.0 Changes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.2.x Beta UI" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.1.0 Changes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.0.0 Baseline" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.8 Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.7 Changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.6 Changes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.5 Changes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.0 Changes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.2.x Beta UI" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.1.0 Changes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.0.0 Baseline" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'v1.3.0 Changes'!$A$4:$E$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'v1.2.x Beta UI'!$A$4:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'v1.1.0 Changes'!$A$4:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'v1.3.0 Changes'!$A$4:$E$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'v1.2.x Beta UI'!$A$4:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'v1.1.0 Changes'!$A$4:$E$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -68,13 +69,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FF6B6B"/>
+      <color rgb="0053D769"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0053D769"/>
+      <color rgb="00FF6B6B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -168,13 +169,13 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -545,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -605,168 +606,190 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>1.3.7</t>
+          <t>1.3.8</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Gain fix + text box + drawing UX</t>
+          <t>Command line + aliases</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Gain slider affects SPL again; sidebar Delete removes all selected speakers; text box annotations (fill + rotate); clean slate on first open; Range off by default; Esc/Line/Shape-menu fixes; command terminal; delay max 10 ms; v1.3.7 Windows Release</t>
+          <t>Command registry (short=full); typed-point DRAW; MOVE/ZOOM sessions; dock/undock terminal; Atomik HELP; Esc keeps float focused; v1.3.8 Windows Release</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>1.3.6</t>
+          <t>1.3.7</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Mic snap + shape-edge tak</t>
+          <t>Gain fix + text box + drawing UX</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Restored original mic Drag::Mic ring snap; tak when drawings meet edge-to-edge; start.md for build/run; v1.3.6 Windows Release</t>
+          <t>Gain slider affects SPL again; sidebar Delete removes all selected speakers; text box annotations (fill + rotate); clean slate on first open; Range off by default; Esc/Line/Shape-menu fixes; command terminal; delay max 10 ms; v1.3.7 Windows Release</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>1.3.5</t>
+          <t>1.3.6</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Mic tool + embedded Q21S Setup</t>
+          <t>Mic snap + shape-edge tak</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Virtual mics, FR floating window, Show Degrees, tak snap sound; Q21S CSVs baked into EXE; Windows Setup without Excel/Data folder</t>
+          <t>Restored original mic Drag::Mic ring snap; tak when drawings meet edge-to-edge; start.md for build/run; v1.3.6 Windows Release</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>1.3.0</t>
+          <t>1.3.5</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Q21S BEM heatmap + Windows/mac product</t>
+          <t>Mic tool + embedded Q21S Setup</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>BEM polar×1/r full-grid SPL, cardioid, Q21S 750×784×917 mm, plot tools/shapes, undo/redo, ATOMIK branding, version archive, Windows portable ZIP (EXE+Data)</t>
+          <t>Virtual mics, FR floating window, Show Degrees, tak snap sound; Q21S CSVs baked into EXE; Windows Setup without Excel/Data folder</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>1.2.x</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>~2026-07</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Beta UI redesign (betav1.2.3)</t>
+          <t>Q21S BEM heatmap + Windows/mac product</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Graph colors.pdf chrome: brand tokens, heatmap colour stops, light/dark sidebar; packaged as betav1.2.3-style Release</t>
+          <t>BEM polar×1/r full-grid SPL, cardioid, Q21S 750×784×917 mm, plot tools/shapes, undo/redo, ATOMIK branding, version archive, Windows portable ZIP (EXE+Data)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>1.1.0</t>
+          <t>1.2.x</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>~2026-07</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Major feature + UX release</t>
+          <t>Beta UI redesign (betav1.2.3)</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Theming, project dashboard/.atmk, heatmap + PDF export, grid/CAD-DXF, array presets, dual datasets, responsive window, branded installer</t>
+          <t>Graph colors.pdf chrome: brand tokens, heatmap colour stops, light/dark sidebar; packaged as betav1.2.3-style Release</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Major feature + UX release</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Theming, project dashboard/.atmk, heatmap + PDF export, grid/CAD-DXF, array presets, dual datasets, responsive window, branded installer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>1.0.0</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Initial baseline</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Dual-subwoofer (XN18) prediction &amp; visualisation in a 30x30 m world; measured directivity added 2026-06-24</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -777,7 +800,480 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Development Timeline</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>What landed when (derived from source history)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Work landed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>v1.0 baseline: engine + UI (Main, MainComponent, ControlPanel, InfoPanel, RadiationPatternComponent, AcousticEngine, ColourMaps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Measured-directivity loading added (MeasurementData)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>v1.1 theming foundation: theme-aware palette + AtomikLookAndFeel (BrandTheme)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Preferences/settings, .atmk projects + dashboard, enhanced heatmap export, PDF pipeline, grid + CAD/DXF, array presets, app icon + installer, header responsiveness, version bump, red-&gt;cyan overhaul</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Window scaling (min size, fixed aspect ratio, clamps); fresh-install guarantee; Recent Projects hygiene</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Dual measurement datasets (Ground Plane / Room), selectable + separate; final naming</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>PS-001…PS-019: 1/3-octave freqs, Ground Plane-only UI, XN18-n, -6 dB legend, PDF/CSV/PNG polish, Set to Default</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>prediction-software repo initial commit (Q21S / XN18 tree)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Plot drawing tools + BEM/directivity math (633fc36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>2026-07 (approx)</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>v1.2.x beta UI redesign (Graph colors.pdf → betav1.2.3 packaging)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>v1.3.0 Windows build: Atomik Simulation Engine rename, ATOMIK-only logo, header v1.3.0 fix, Ctrl+Z/Y, Statistics button, single Release exe</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Q21S BEM polar×1/r, cardioid, cabinet size, heatmap docs, version archive; plot shapes + opacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Windows Q21S data-path fix + portable ZIP (EXE+MeasurementIntegrationPack); archive Windows = ZIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>v1.3.8  -  Detailed Changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04  |  Command line aliases + typed points + MOVE/ZOOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Command registry</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Short form and full name share one handler (L/LINE, PE/PENCIL, SPK/ADDSPEAKER, …)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Typed-point DRAW</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>After LINE/CIRCLE/… enter x,y (metres) or click the plot</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>MOVE / ZOOM sessions</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>MOVE base/second point; ZOOM [Extents/In/Out]</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Dock / Undock</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Floating terminal window; state remembered</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>HELP / ?</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Atomik-branded command list (no third-party CAD branding)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Undocked Esc / finish</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Completing or cancelling a command no longer loses the floating terminal</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Version → v1.3.8</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>App, resource, archive HTML/json, Windows Release EXE</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -840,7 +1336,7 @@
           <t>Speakers</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -867,7 +1363,7 @@
           <t>Speakers</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -894,7 +1390,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -921,7 +1417,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -948,7 +1444,7 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -975,7 +1471,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1002,7 +1498,7 @@
           <t>Speakers</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1056,7 +1552,7 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1113,7 +1609,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1176,7 +1672,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -1203,7 +1699,7 @@
           <t>Plot Snap</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -1230,7 +1726,7 @@
           <t>Docs</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1287,7 +1783,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1350,7 +1846,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1377,7 +1873,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1404,7 +1900,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1431,7 +1927,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1458,7 +1954,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1485,7 +1981,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1512,7 +2008,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1542,7 +2038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1620,7 +2116,7 @@
           <t>Engine</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1647,7 +2143,7 @@
           <t>Array presets</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1674,7 +2170,7 @@
           <t>Docs / pack</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1701,7 +2197,7 @@
           <t>Archive</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1728,7 +2224,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1755,7 +2251,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1782,7 +2278,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1809,7 +2305,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1836,7 +2332,7 @@
           <t>Editing</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1863,7 +2359,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1890,7 +2386,7 @@
           <t>DSP / UI (PS batch)</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1944,7 +2440,7 @@
           <t>Engine</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1998,7 +2494,7 @@
           <t>Measurement</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2052,7 +2548,7 @@
           <t>Branding</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2106,7 +2602,7 @@
           <t>Measurement</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2160,7 +2656,7 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2187,7 +2683,7 @@
           <t>Engine</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2214,7 +2710,7 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2241,7 +2737,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2268,7 +2764,7 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2313,7 +2809,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2376,7 +2872,7 @@
           <t>Brand</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2430,7 +2926,7 @@
           <t>Heatmap</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2484,7 +2980,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2515,7 +3011,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2593,7 +3089,7 @@
           <t>Theming &amp; Preferences</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2620,7 +3116,7 @@
           <t>Theming &amp; Preferences</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2647,7 +3143,7 @@
           <t>Theming &amp; Preferences</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2674,7 +3170,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2701,7 +3197,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2728,7 +3224,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2755,7 +3251,7 @@
           <t>Heatmap Export</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2782,7 +3278,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2809,7 +3305,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2836,7 +3332,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2863,7 +3359,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2890,7 +3386,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2917,7 +3413,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2944,7 +3440,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2971,7 +3467,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2998,7 +3494,7 @@
           <t>Array Presets</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3025,7 +3521,7 @@
           <t>Array Presets</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3052,7 +3548,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3079,7 +3575,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3106,7 +3602,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3133,7 +3629,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3160,7 +3656,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3187,7 +3683,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3214,7 +3710,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3241,7 +3737,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3268,7 +3764,7 @@
           <t>Branding &amp; Installer</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3295,7 +3791,7 @@
           <t>Branding &amp; Installer</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -3349,7 +3845,7 @@
           <t>Color system</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -3403,7 +3899,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -3430,7 +3926,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3457,7 +3953,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3484,7 +3980,7 @@
           <t>Recent Projects</t>
         </is>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3511,7 +4007,7 @@
           <t>Installer</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3556,7 +4052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3748,222 +4244,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Development Timeline</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>What landed when (derived from source history)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Work landed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>v1.0 baseline: engine + UI (Main, MainComponent, ControlPanel, InfoPanel, RadiationPatternComponent, AcousticEngine, ColourMaps)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Measured-directivity loading added (MeasurementData)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>v1.1 theming foundation: theme-aware palette + AtomikLookAndFeel (BrandTheme)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Preferences/settings, .atmk projects + dashboard, enhanced heatmap export, PDF pipeline, grid + CAD/DXF, array presets, app icon + installer, header responsiveness, version bump, red-&gt;cyan overhaul</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Window scaling (min size, fixed aspect ratio, clamps); fresh-install guarantee; Recent Projects hygiene</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Dual measurement datasets (Ground Plane / Room), selectable + separate; final naming</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>PS-001…PS-019: 1/3-octave freqs, Ground Plane-only UI, XN18-n, -6 dB legend, PDF/CSV/PNG polish, Set to Default</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>prediction-software repo initial commit (Q21S / XN18 tree)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Plot drawing tools + BEM/directivity math (633fc36)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>2026-07 (approx)</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>v1.2.x beta UI redesign (Graph colors.pdf → betav1.2.3 packaging)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>v1.3.0 Windows build: Atomik Simulation Engine rename, ATOMIK-only logo, header v1.3.0 fix, Ctrl+Z/Y, Statistics button, single Release exe</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Q21S BEM polar×1/r, cardioid, cabinet size, heatmap docs, version archive; plot shapes + opacity</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Windows Q21S data-path fix + portable ZIP (EXE+MeasurementIntegrationPack); archive Windows = ZIP</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Lighten the plot grid; refresh the v1.4.0.1 build
The light theme's plotGrid token is an opaque mid-grey intended for a pale
canvas. Drawn at full strength over the near-black SPL field it overpowered
the data: major lines were at 100% alpha and minors at 45%. Now 42% and 16%.

Both alphas and both line thicknesses moved into UiConfig::PlotGrid, so the
grid's prominence is a single edit rather than four literals buried in
drawGrid.

Rebuilds the v1.4.0.1 EXE and source zip in place (no version bump), and adds
the change to the existing 1.4.0.1 sections of CHANGELOG.md and
CHANGELOG.xlsx and to its archive entry. Earlier entries are untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ShyamGui/CHANGELOG.xlsx
+++ b/ShyamGui/CHANGELOG.xlsx
@@ -174,10 +174,10 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -623,7 +623,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Fill-the-canvas fit is the zoom floor, so the plot never letterboxes; pan fixed and middle-drag pans from any tool; Q21S cabinet corrected to 1546 x 679 x 1024 mm and drawn to scale; SPL caption back at the canvas edge</t>
+          <t>Fill-the-canvas fit is the zoom floor, so the plot never letterboxes; pan fixed and middle-drag pans from any tool; Q21S cabinet corrected to 1546 x 679 x 1024 mm and drawn to scale; SPL caption back at the canvas edge; lighter grid lines</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -1810,7 +1810,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -1837,7 +1837,7 @@
           <t>Recent Projects</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -1864,7 +1864,7 @@
           <t>Installer</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2327,7 +2327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2492,19 +2492,19 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Fixed</t>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Changed</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Pan did nothing</t>
+          <t>Grid lines lighter over the field</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>The view offset was clamped back to zero on every drag. Panning now moves the view across the field with no re-solve, so it is instant and placement is exact</t>
+          <t>The light theme's opaque plotGrid overpowered the near-black field: major lines 100% -&gt; 42% alpha, minor 45% -&gt; 16%. Weights and thicknesses collected in UiConfig::PlotGrid</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -2519,19 +2519,19 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Zoom anchored on the field corner</t>
+          <t>Pan did nothing</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Zooming in walked off into empty space; it now holds the view centre</t>
+          <t>The view offset was clamped back to zero on every drag. Panning now moves the view across the field with no re-solve, so it is instant and placement is exact</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -2543,25 +2543,52 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>Plot</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Zoom anchored on the field corner</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Zooming in walked off into empty space; it now holds the view centre</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Version -&gt; v1.4.0.1</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>App, resource, installer, archive HTML/json, Windows Release EXE</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
@@ -2774,7 +2801,7 @@
           <t>Speakers</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2801,7 +2828,7 @@
           <t>Speakers</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2990,7 +3017,7 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3017,7 +3044,7 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3044,7 +3071,7 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3071,7 +3098,7 @@
           <t>Measurements</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3098,7 +3125,7 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3125,7 +3152,7 @@
           <t>Help</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3152,7 +3179,7 @@
           <t>Ribbon</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3179,7 +3206,7 @@
           <t>Legend</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3206,7 +3233,7 @@
           <t>Plot</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3233,7 +3260,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3488,7 +3515,7 @@
           <t>Terminal</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3608,7 +3635,7 @@
           <t>Speakers</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3635,7 +3662,7 @@
           <t>Speakers</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3662,7 +3689,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3689,7 +3716,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3944,7 +3971,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3971,7 +3998,7 @@
           <t>Plot Snap</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -4955,7 +4982,7 @@
           <t>Engine</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -4982,7 +5009,7 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -5009,7 +5036,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -5036,7 +5063,7 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>

</xml_diff>